<commit_message>
corrected age input variable
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="259" documentId="8_{5005C4B8-8269-4712-9267-05709C8265AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{339FDDB2-46A3-461B-A141-A096D22A068A}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="8_{5005C4B8-8269-4712-9267-05709C8265AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3C1AF40-C97F-4DEB-8AE0-57A346E08889}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
@@ -1270,10 +1270,6 @@
     <t>dt12getoplcs1; ha12howgtstr7</t>
   </si>
   <si>
-    <t xml:space="preserve">r12dintvwrage
-</t>
-  </si>
-  <si>
     <t>R12 AB COVER DATE MONTH;
 R12 AB COVER DATE YEAR</t>
   </si>
@@ -1636,6 +1632,9 @@
 dt12getoplcs1 == 2 &amp; ha12howgtstr7 == 2 ~ 0;
 TRUE ~ NA_integer_
 )</t>
+  </si>
+  <si>
+    <t>r12dintvwrage</t>
   </si>
 </sst>
 </file>
@@ -2173,7 +2172,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>3</v>
@@ -2182,10 +2181,10 @@
         <v>4</v>
       </c>
       <c r="G1" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="H1" s="12" t="s">
         <v>367</v>
-      </c>
-      <c r="H1" s="12" t="s">
-        <v>368</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>1</v>
@@ -2197,10 +2196,10 @@
         <v>275</v>
       </c>
       <c r="L1" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="M1" s="10" t="s">
         <v>369</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>370</v>
       </c>
       <c r="N1" s="13" t="s">
         <v>277</v>
@@ -2215,7 +2214,7 @@
         <v>280</v>
       </c>
       <c r="R1" s="10" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="S1" s="14" t="s">
         <v>9</v>
@@ -2259,7 +2258,7 @@
         <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J2" t="s">
         <v>284</v>
@@ -2279,7 +2278,7 @@
         <v>311</v>
       </c>
       <c r="Q2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="R2" s="16"/>
       <c r="S2" s="4"/>
@@ -2290,7 +2289,7 @@
         <v>27</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="X2" s="4" t="s">
         <v>284</v>
@@ -2317,7 +2316,7 @@
         <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J3" t="s">
         <v>292</v>
@@ -2328,7 +2327,7 @@
       </c>
       <c r="O3" s="16"/>
       <c r="Q3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
@@ -2370,13 +2369,13 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>316</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
@@ -2399,7 +2398,7 @@
         <v>14</v>
       </c>
       <c r="Y4" s="11" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
@@ -2425,13 +2424,13 @@
         <v>25</v>
       </c>
       <c r="I5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="K5" t="s">
         <v>400</v>
-      </c>
-      <c r="K5" t="s">
-        <v>401</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>286</v>
@@ -2445,7 +2444,7 @@
         <v>311</v>
       </c>
       <c r="Q5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U5" t="s">
         <v>26</v>
@@ -2484,13 +2483,13 @@
       </c>
       <c r="H6" s="2"/>
       <c r="I6" t="s">
-        <v>378</v>
-      </c>
-      <c r="J6" t="s">
-        <v>336</v>
+        <v>377</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>404</v>
       </c>
       <c r="K6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="5" t="s">
@@ -2504,7 +2503,7 @@
         <v>311</v>
       </c>
       <c r="Q6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R6" t="s">
         <v>32</v>
@@ -2545,7 +2544,7 @@
         <v>36</v>
       </c>
       <c r="I7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J7" t="s">
         <v>292</v>
@@ -2596,13 +2595,13 @@
         <v>42</v>
       </c>
       <c r="I8" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J8" t="s">
         <v>317</v>
       </c>
       <c r="K8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>291</v>
@@ -2616,7 +2615,7 @@
         <v>311</v>
       </c>
       <c r="Q8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U8" t="s">
         <v>26</v>
@@ -2654,13 +2653,13 @@
         <v>46</v>
       </c>
       <c r="I9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J9" t="s">
         <v>318</v>
       </c>
       <c r="K9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>302</v>
@@ -2674,7 +2673,7 @@
         <v>311</v>
       </c>
       <c r="Q9" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U9" s="4" t="s">
         <v>26</v>
@@ -2686,7 +2685,7 @@
         <v>51</v>
       </c>
       <c r="X9" s="11" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -2709,13 +2708,13 @@
         <v>50</v>
       </c>
       <c r="I10" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J10" t="s">
         <v>319</v>
       </c>
       <c r="K10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="N10" t="s">
         <v>315</v>
@@ -2725,7 +2724,7 @@
         <v>311</v>
       </c>
       <c r="Q10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R10" t="s">
         <v>293</v>
@@ -2763,13 +2762,13 @@
         <v>13</v>
       </c>
       <c r="I11" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J11" t="s">
+        <v>373</v>
+      </c>
+      <c r="K11" t="s">
         <v>374</v>
-      </c>
-      <c r="K11" t="s">
-        <v>375</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>13</v>
@@ -2782,7 +2781,7 @@
         <v>311</v>
       </c>
       <c r="Q11" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U11" t="s">
         <v>26</v>
@@ -2820,13 +2819,13 @@
         <v>58</v>
       </c>
       <c r="I12" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J12" t="s">
         <v>317</v>
       </c>
       <c r="K12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="L12" t="s">
         <v>291</v>
@@ -2840,7 +2839,7 @@
         <v>311</v>
       </c>
       <c r="Q12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U12" t="s">
         <v>26</v>
@@ -2852,7 +2851,7 @@
         <v>38</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="171" x14ac:dyDescent="0.45">
@@ -2878,13 +2877,13 @@
         <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J13" t="s">
         <v>320</v>
       </c>
       <c r="K13" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>294</v>
@@ -2933,13 +2932,13 @@
         <v>66</v>
       </c>
       <c r="I14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J14" t="s">
         <v>320</v>
       </c>
       <c r="K14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>294</v>
@@ -2953,7 +2952,7 @@
         <v>311</v>
       </c>
       <c r="Q14" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U14" t="s">
         <v>26</v>
@@ -2965,7 +2964,7 @@
         <v>38</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -2991,16 +2990,16 @@
         <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J15" t="s">
+        <v>385</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="L15" s="5" t="s">
         <v>386</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>387</v>
       </c>
       <c r="N15" t="s">
         <v>315</v>
@@ -3010,7 +3009,7 @@
         <v>311</v>
       </c>
       <c r="Q15" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U15" s="4" t="s">
         <v>14</v>
@@ -3025,7 +3024,7 @@
         <v>14</v>
       </c>
       <c r="Y15" s="11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
@@ -3052,13 +3051,13 @@
       </c>
       <c r="H16" s="2"/>
       <c r="I16" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>321</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>297</v>
@@ -3071,7 +3070,7 @@
         <v>311</v>
       </c>
       <c r="Q16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R16" t="s">
         <v>296</v>
@@ -3086,7 +3085,7 @@
         <v>75</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
@@ -3112,7 +3111,7 @@
         <v>78</v>
       </c>
       <c r="I17" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J17" t="s">
         <v>292</v>
@@ -3125,7 +3124,7 @@
         <v>311</v>
       </c>
       <c r="Q17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U17" s="4" t="s">
         <v>26</v>
@@ -3164,13 +3163,13 @@
       </c>
       <c r="H18" s="2"/>
       <c r="I18" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J18" t="s">
         <v>322</v>
       </c>
       <c r="K18" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="N18" t="s">
         <v>315</v>
@@ -3180,7 +3179,7 @@
         <v>311</v>
       </c>
       <c r="Q18" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R18" t="s">
         <v>82</v>
@@ -3195,7 +3194,7 @@
         <v>75</v>
       </c>
       <c r="X18" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
@@ -3221,7 +3220,7 @@
         <v>78</v>
       </c>
       <c r="I19" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J19" t="s">
         <v>292</v>
@@ -3234,7 +3233,7 @@
         <v>311</v>
       </c>
       <c r="Q19" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U19" s="4" t="s">
         <v>26</v>
@@ -3272,13 +3271,13 @@
         <v>87</v>
       </c>
       <c r="I20" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>323</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="N20" t="s">
         <v>315</v>
@@ -3288,7 +3287,7 @@
         <v>311</v>
       </c>
       <c r="Q20" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R20" t="s">
         <v>299</v>
@@ -3303,7 +3302,7 @@
         <v>51</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="15.75" x14ac:dyDescent="0.45">
@@ -3330,13 +3329,13 @@
       </c>
       <c r="H21" s="2"/>
       <c r="I21" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J21" t="s">
         <v>324</v>
       </c>
       <c r="K21" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="N21" t="s">
         <v>315</v>
@@ -3346,7 +3345,7 @@
         <v>311</v>
       </c>
       <c r="Q21" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R21" t="s">
         <v>74</v>
@@ -3361,7 +3360,7 @@
         <v>75</v>
       </c>
       <c r="X21" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="57" x14ac:dyDescent="0.45">
@@ -3387,13 +3386,13 @@
         <v>78</v>
       </c>
       <c r="I22" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J22" t="s">
         <v>325</v>
       </c>
       <c r="K22" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>300</v>
@@ -3407,7 +3406,7 @@
         <v>311</v>
       </c>
       <c r="Q22" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U22" t="s">
         <v>26</v>
@@ -3445,7 +3444,7 @@
         <v>94</v>
       </c>
       <c r="I23" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J23" t="s">
         <v>292</v>
@@ -3478,7 +3477,7 @@
         <v>13</v>
       </c>
       <c r="I24" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J24" t="s">
         <v>292</v>
@@ -3523,7 +3522,7 @@
         <v>100</v>
       </c>
       <c r="I25" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J25" t="s">
         <v>292</v>
@@ -3568,7 +3567,7 @@
         <v>100</v>
       </c>
       <c r="I26" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J26" t="s">
         <v>292</v>
@@ -3613,7 +3612,7 @@
         <v>106</v>
       </c>
       <c r="I27" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J27" t="s">
         <v>292</v>
@@ -3659,7 +3658,7 @@
       </c>
       <c r="H28" s="2"/>
       <c r="I28" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J28" t="s">
         <v>292</v>
@@ -3704,7 +3703,7 @@
         <v>112</v>
       </c>
       <c r="I29" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J29" t="s">
         <v>292</v>
@@ -3749,7 +3748,7 @@
         <v>115</v>
       </c>
       <c r="I30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J30" t="s">
         <v>292</v>
@@ -3794,7 +3793,7 @@
         <v>118</v>
       </c>
       <c r="I31" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J31" t="s">
         <v>292</v>
@@ -3839,7 +3838,7 @@
         <v>121</v>
       </c>
       <c r="I32" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J32" t="s">
         <v>292</v>
@@ -3884,7 +3883,7 @@
         <v>121</v>
       </c>
       <c r="I33" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J33" t="s">
         <v>292</v>
@@ -3929,7 +3928,7 @@
         <v>121</v>
       </c>
       <c r="I34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J34" t="s">
         <v>292</v>
@@ -3974,7 +3973,7 @@
         <v>121</v>
       </c>
       <c r="I35" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J35" t="s">
         <v>292</v>
@@ -4019,7 +4018,7 @@
         <v>121</v>
       </c>
       <c r="I36" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J36" t="s">
         <v>292</v>
@@ -4064,7 +4063,7 @@
         <v>132</v>
       </c>
       <c r="I37" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J37" t="s">
         <v>292</v>
@@ -4110,7 +4109,7 @@
       </c>
       <c r="H38" s="2"/>
       <c r="I38" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J38" t="s">
         <v>292</v>
@@ -4155,7 +4154,7 @@
         <v>140</v>
       </c>
       <c r="I39" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J39" t="s">
         <v>292</v>
@@ -4207,7 +4206,7 @@
       </c>
       <c r="H40" s="2"/>
       <c r="I40" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J40" t="s">
         <v>292</v>
@@ -4252,7 +4251,7 @@
         <v>140</v>
       </c>
       <c r="I41" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J41" t="s">
         <v>292</v>
@@ -4297,7 +4296,7 @@
         <v>149</v>
       </c>
       <c r="I42" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J42" t="s">
         <v>292</v>
@@ -4343,7 +4342,7 @@
       </c>
       <c r="H43" s="2"/>
       <c r="I43" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J43" t="s">
         <v>292</v>
@@ -4388,7 +4387,7 @@
         <v>156</v>
       </c>
       <c r="I44" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J44" t="s">
         <v>292</v>
@@ -4433,13 +4432,13 @@
         <v>160</v>
       </c>
       <c r="I45" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J45" t="s">
         <v>326</v>
       </c>
       <c r="K45" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>302</v>
@@ -4489,7 +4488,7 @@
         <v>163</v>
       </c>
       <c r="I46" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J46" t="s">
         <v>327</v>
@@ -4542,13 +4541,13 @@
       </c>
       <c r="H47" s="2"/>
       <c r="I47" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J47" t="s">
         <v>327</v>
       </c>
       <c r="K47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>165</v>
@@ -4562,7 +4561,7 @@
         <v>311</v>
       </c>
       <c r="Q47" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U47" t="s">
         <v>26</v>
@@ -4574,7 +4573,7 @@
         <v>51</v>
       </c>
       <c r="X47" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="48" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
@@ -4600,13 +4599,13 @@
         <v>171</v>
       </c>
       <c r="I48" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J48" t="s">
         <v>328</v>
       </c>
       <c r="K48" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="L48" s="5" t="s">
         <v>305</v>
@@ -4620,7 +4619,7 @@
         <v>311</v>
       </c>
       <c r="Q48" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U48" t="s">
         <v>26</v>
@@ -4632,10 +4631,10 @@
         <v>38</v>
       </c>
       <c r="X48" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="Y48" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="49" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
@@ -4661,13 +4660,13 @@
         <v>175</v>
       </c>
       <c r="I49" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J49" t="s">
         <v>329</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>306</v>
@@ -4681,7 +4680,7 @@
         <v>311</v>
       </c>
       <c r="Q49" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S49" s="2"/>
       <c r="U49" t="s">
@@ -4694,10 +4693,10 @@
         <v>51</v>
       </c>
       <c r="X49" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="Y49" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="50" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
@@ -4723,13 +4722,13 @@
         <v>175</v>
       </c>
       <c r="I50" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J50" t="s">
         <v>330</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>306</v>
@@ -4743,7 +4742,7 @@
         <v>311</v>
       </c>
       <c r="Q50" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S50" s="2"/>
       <c r="U50" t="s">
@@ -4756,10 +4755,10 @@
         <v>51</v>
       </c>
       <c r="X50" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="51" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
@@ -4785,13 +4784,13 @@
         <v>175</v>
       </c>
       <c r="I51" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J51" t="s">
         <v>331</v>
       </c>
       <c r="K51" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>182</v>
@@ -4805,7 +4804,7 @@
         <v>311</v>
       </c>
       <c r="Q51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U51" t="s">
         <v>26</v>
@@ -4817,7 +4816,7 @@
         <v>51</v>
       </c>
       <c r="X51" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="52" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
@@ -4843,7 +4842,7 @@
         <v>186</v>
       </c>
       <c r="I52" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J52" t="s">
         <v>292</v>
@@ -4890,13 +4889,13 @@
         <v>175</v>
       </c>
       <c r="I53" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>332</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>307</v>
@@ -4910,7 +4909,7 @@
         <v>311</v>
       </c>
       <c r="Q53" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U53" t="s">
         <v>26</v>
@@ -4922,7 +4921,7 @@
         <v>51</v>
       </c>
       <c r="X53" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="54" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -4948,7 +4947,7 @@
         <v>175</v>
       </c>
       <c r="I54" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J54" t="s">
         <v>292</v>
@@ -4993,7 +4992,7 @@
         <v>175</v>
       </c>
       <c r="I55" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J55" t="s">
         <v>292</v>
@@ -5040,7 +5039,7 @@
         <v>175</v>
       </c>
       <c r="I56" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J56" t="s">
         <v>292</v>
@@ -5087,7 +5086,7 @@
         <v>175</v>
       </c>
       <c r="I57" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J57" t="s">
         <v>292</v>
@@ -5132,7 +5131,7 @@
         <v>175</v>
       </c>
       <c r="I58" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J58" t="s">
         <v>292</v>
@@ -5174,7 +5173,7 @@
         <v>16</v>
       </c>
       <c r="I59" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J59" t="s">
         <v>292</v>
@@ -5216,7 +5215,7 @@
         <v>16</v>
       </c>
       <c r="I60" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J60" t="s">
         <v>292</v>
@@ -5258,7 +5257,7 @@
         <v>16</v>
       </c>
       <c r="I61" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J61" t="s">
         <v>292</v>
@@ -5300,7 +5299,7 @@
         <v>16</v>
       </c>
       <c r="I62" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J62" t="s">
         <v>292</v>
@@ -5342,7 +5341,7 @@
         <v>16</v>
       </c>
       <c r="I63" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J63" t="s">
         <v>292</v>
@@ -5386,7 +5385,7 @@
         <v>16</v>
       </c>
       <c r="I64" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J64" t="s">
         <v>292</v>
@@ -5429,7 +5428,7 @@
       </c>
       <c r="H65" s="2"/>
       <c r="I65" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J65" t="s">
         <v>292</v>
@@ -5474,16 +5473,16 @@
         <v>216</v>
       </c>
       <c r="I66" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J66" t="s">
         <v>333</v>
       </c>
       <c r="K66" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="M66" s="5"/>
       <c r="N66" t="s">
@@ -5494,7 +5493,7 @@
         <v>311</v>
       </c>
       <c r="Q66" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S66" s="2"/>
       <c r="U66" t="s">
@@ -5507,7 +5506,7 @@
         <v>38</v>
       </c>
       <c r="X66" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="Y66" s="2"/>
     </row>
@@ -5535,7 +5534,7 @@
       </c>
       <c r="H67" s="2"/>
       <c r="I67" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J67" t="s">
         <v>292</v>
@@ -5580,7 +5579,7 @@
         <v>222</v>
       </c>
       <c r="I68" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J68" t="s">
         <v>292</v>
@@ -5625,13 +5624,13 @@
         <v>225</v>
       </c>
       <c r="I69" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J69" t="s">
         <v>334</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>308</v>
@@ -5645,7 +5644,7 @@
         <v>311</v>
       </c>
       <c r="Q69" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U69" t="s">
         <v>26</v>
@@ -5657,7 +5656,7 @@
         <v>51</v>
       </c>
       <c r="X69" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="70" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
@@ -5683,7 +5682,7 @@
         <v>228</v>
       </c>
       <c r="I70" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J70" t="s">
         <v>292</v>
@@ -5728,7 +5727,7 @@
         <v>228</v>
       </c>
       <c r="I71" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J71" t="s">
         <v>292</v>
@@ -5771,7 +5770,7 @@
       </c>
       <c r="H72" s="2"/>
       <c r="I72" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J72" t="s">
         <v>292</v>
@@ -5816,7 +5815,7 @@
         <v>236</v>
       </c>
       <c r="I73" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J73" t="s">
         <v>292</v>
@@ -5861,7 +5860,7 @@
         <v>240</v>
       </c>
       <c r="I74" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J74" t="s">
         <v>292</v>
@@ -5906,7 +5905,7 @@
         <v>244</v>
       </c>
       <c r="I75" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J75" t="s">
         <v>292</v>
@@ -5952,7 +5951,7 @@
       </c>
       <c r="H76" s="2"/>
       <c r="I76" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J76" t="s">
         <v>292</v>
@@ -5999,7 +5998,7 @@
         <v>251</v>
       </c>
       <c r="I77" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J77" t="s">
         <v>292</v>
@@ -6044,7 +6043,7 @@
         <v>255</v>
       </c>
       <c r="I78" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J78" t="s">
         <v>292</v>
@@ -6089,7 +6088,7 @@
         <v>258</v>
       </c>
       <c r="I79" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J79" t="s">
         <v>292</v>
@@ -6134,13 +6133,13 @@
         <v>175</v>
       </c>
       <c r="I80" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J80" t="s">
+        <v>388</v>
+      </c>
+      <c r="K80" t="s">
         <v>389</v>
-      </c>
-      <c r="K80" t="s">
-        <v>390</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>310</v>
@@ -6154,7 +6153,7 @@
         <v>311</v>
       </c>
       <c r="Q80" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S80" s="2"/>
       <c r="U80" t="s">
@@ -6167,10 +6166,10 @@
         <v>51</v>
       </c>
       <c r="X80" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="Y80" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="81" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
@@ -6196,13 +6195,13 @@
         <v>175</v>
       </c>
       <c r="I81" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J81" t="s">
         <v>335</v>
       </c>
       <c r="K81" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>309</v>
@@ -6216,7 +6215,7 @@
         <v>311</v>
       </c>
       <c r="Q81" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="U81" t="s">
         <v>26</v>
@@ -6228,7 +6227,7 @@
         <v>51</v>
       </c>
       <c r="X81" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="82" spans="1:25" ht="409.5" x14ac:dyDescent="0.45">
@@ -6254,16 +6253,16 @@
         <v>175</v>
       </c>
       <c r="I82" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J82" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="K82" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="K82" s="2" t="s">
+      <c r="L82" s="5" t="s">
         <v>394</v>
-      </c>
-      <c r="L82" s="5" t="s">
-        <v>395</v>
       </c>
       <c r="M82" s="5"/>
       <c r="N82" t="s">
@@ -6274,7 +6273,7 @@
         <v>311</v>
       </c>
       <c r="Q82" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S82" s="2"/>
       <c r="U82" t="s">
@@ -6287,10 +6286,10 @@
         <v>38</v>
       </c>
       <c r="X82" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="Y82" s="2" t="s">
         <v>396</v>
-      </c>
-      <c r="Y82" s="2" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="83" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -6313,7 +6312,7 @@
         <v>50</v>
       </c>
       <c r="I83" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J83" s="2" t="s">
         <v>292</v>
@@ -6358,7 +6357,7 @@
         <v>274</v>
       </c>
       <c r="I84" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J84" s="2" t="s">
         <v>292</v>

</xml_diff>

<commit_message>
r13 correction of algorithms
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{B04BC2F6-0886-423B-9CF8-2AF8452D03D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32DD84DE-0198-46E0-8A8F-FA88CCBB9112}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{B04BC2F6-0886-423B-9CF8-2AF8452D03D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3921F31C-8E7E-479F-8418-8CCBAC8E8062}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="401">
   <si>
     <t>index</t>
   </si>
@@ -1152,10 +1152,6 @@
   <si>
     <t>R13 AB COVER DATE MONTH;
 R13 AB COVER DATE YEAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r13dintvwrage
-</t>
   </si>
   <si>
     <t>R13 D AGE OF SP AT INTERVIEW</t>
@@ -1541,6 +1537,9 @@
 dt13getoplcs1 == 2 &amp; ha13howgtstr7 == 2 ~ 0;
 TRUE ~ NA_integer_
 )</t>
+  </si>
+  <si>
+    <t>r13dintvwrage</t>
   </si>
 </sst>
 </file>
@@ -1663,7 +1662,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1703,11 +1702,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2169,7 +2163,7 @@
         <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J2" t="s">
         <v>282</v>
@@ -2182,14 +2176,14 @@
       </c>
       <c r="M2"/>
       <c r="N2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O2" s="16"/>
       <c r="P2" t="s">
         <v>309</v>
       </c>
       <c r="Q2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="R2" s="16"/>
       <c r="S2" s="4"/>
@@ -2227,18 +2221,18 @@
         <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J3" t="s">
         <v>290</v>
       </c>
       <c r="K3"/>
       <c r="N3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O3" s="16"/>
       <c r="Q3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
@@ -2280,7 +2274,7 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>321</v>
@@ -2291,7 +2285,7 @@
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
       <c r="N4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O4" s="16"/>
       <c r="R4" s="4"/>
@@ -2335,27 +2329,27 @@
         <v>24</v>
       </c>
       <c r="I5" t="s">
+        <v>376</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" t="s">
         <v>378</v>
-      </c>
-      <c r="K5" t="s">
-        <v>379</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>284</v>
       </c>
       <c r="M5" s="5"/>
       <c r="N5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" t="s">
         <v>309</v>
       </c>
       <c r="Q5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U5" t="s">
         <v>25</v>
@@ -2394,25 +2388,27 @@
       </c>
       <c r="H6" s="2"/>
       <c r="I6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="K6" t="s">
         <v>323</v>
       </c>
-      <c r="K6" t="s">
-        <v>324</v>
-      </c>
       <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="M6" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="N6" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O6" s="16"/>
       <c r="P6" t="s">
         <v>309</v>
       </c>
       <c r="Q6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R6" t="s">
         <v>31</v>
@@ -2453,7 +2449,7 @@
         <v>35</v>
       </c>
       <c r="I7" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J7" t="s">
         <v>290</v>
@@ -2461,7 +2457,7 @@
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O7" s="16"/>
       <c r="S7" s="2"/>
@@ -2504,27 +2500,27 @@
         <v>41</v>
       </c>
       <c r="I8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J8" t="s">
+        <v>324</v>
+      </c>
+      <c r="K8" t="s">
         <v>325</v>
-      </c>
-      <c r="K8" t="s">
-        <v>326</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>289</v>
       </c>
       <c r="M8" s="5"/>
       <c r="N8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O8" s="16"/>
       <c r="P8" t="s">
         <v>309</v>
       </c>
       <c r="Q8" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U8" t="s">
         <v>25</v>
@@ -2562,27 +2558,27 @@
         <v>45</v>
       </c>
       <c r="I9" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J9" t="s">
+        <v>326</v>
+      </c>
+      <c r="K9" t="s">
         <v>327</v>
-      </c>
-      <c r="K9" t="s">
-        <v>328</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>300</v>
       </c>
       <c r="M9" s="5"/>
       <c r="N9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O9" s="16"/>
       <c r="P9" t="s">
         <v>309</v>
       </c>
       <c r="Q9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U9" s="4" t="s">
         <v>25</v>
@@ -2594,7 +2590,7 @@
         <v>50</v>
       </c>
       <c r="X9" s="11" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -2617,23 +2613,23 @@
         <v>49</v>
       </c>
       <c r="I10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J10" t="s">
+        <v>328</v>
+      </c>
+      <c r="K10" t="s">
         <v>329</v>
       </c>
-      <c r="K10" t="s">
-        <v>330</v>
-      </c>
       <c r="N10" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O10" s="16"/>
       <c r="P10" t="s">
         <v>309</v>
       </c>
       <c r="Q10" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R10" t="s">
         <v>291</v>
@@ -2671,26 +2667,26 @@
         <v>13</v>
       </c>
       <c r="I11" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J11" t="s">
+        <v>330</v>
+      </c>
+      <c r="K11" t="s">
         <v>331</v>
-      </c>
-      <c r="K11" t="s">
-        <v>332</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="N11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O11" s="16"/>
       <c r="P11" t="s">
         <v>309</v>
       </c>
       <c r="Q11" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U11" t="s">
         <v>25</v>
@@ -2728,27 +2724,27 @@
         <v>57</v>
       </c>
       <c r="I12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J12" t="s">
+        <v>324</v>
+      </c>
+      <c r="K12" t="s">
         <v>325</v>
-      </c>
-      <c r="K12" t="s">
-        <v>326</v>
       </c>
       <c r="L12" t="s">
         <v>289</v>
       </c>
       <c r="M12"/>
       <c r="N12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O12" s="16"/>
       <c r="P12" t="s">
         <v>309</v>
       </c>
       <c r="Q12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U12" t="s">
         <v>25</v>
@@ -2760,7 +2756,7 @@
         <v>37</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="171" x14ac:dyDescent="0.45">
@@ -2786,20 +2782,20 @@
         <v>61</v>
       </c>
       <c r="I13" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J13" t="s">
+        <v>332</v>
+      </c>
+      <c r="K13" t="s">
         <v>333</v>
-      </c>
-      <c r="K13" t="s">
-        <v>334</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>292</v>
       </c>
       <c r="M13" s="5"/>
       <c r="N13" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O13" s="16"/>
       <c r="U13" t="s">
@@ -2841,27 +2837,27 @@
         <v>65</v>
       </c>
       <c r="I14" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J14" t="s">
+        <v>332</v>
+      </c>
+      <c r="K14" t="s">
         <v>333</v>
-      </c>
-      <c r="K14" t="s">
-        <v>334</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>292</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O14" s="16"/>
       <c r="P14" t="s">
         <v>309</v>
       </c>
       <c r="Q14" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U14" t="s">
         <v>25</v>
@@ -2873,7 +2869,7 @@
         <v>37</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -2899,24 +2895,23 @@
         <v>68</v>
       </c>
       <c r="I15" t="s">
-        <v>377</v>
-      </c>
-      <c r="J15" s="18" t="s">
-        <v>387</v>
+        <v>376</v>
+      </c>
+      <c r="J15" t="s">
+        <v>386</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="L15" s="19"/>
+        <v>334</v>
+      </c>
       <c r="N15" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O15" s="16"/>
       <c r="P15" t="s">
         <v>309</v>
       </c>
       <c r="Q15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U15" s="4" t="s">
         <v>14</v>
@@ -2930,8 +2925,8 @@
       <c r="X15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="Y15" s="17" t="s">
-        <v>386</v>
+      <c r="Y15" s="11" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
@@ -2958,26 +2953,26 @@
       </c>
       <c r="H16" s="2"/>
       <c r="I16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J16" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>337</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>295</v>
       </c>
       <c r="N16" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O16" s="16"/>
       <c r="P16" t="s">
         <v>309</v>
       </c>
       <c r="Q16" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R16" t="s">
         <v>294</v>
@@ -2992,7 +2987,7 @@
         <v>74</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
@@ -3018,20 +3013,20 @@
         <v>77</v>
       </c>
       <c r="I17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J17" t="s">
         <v>290</v>
       </c>
       <c r="N17" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O17" s="16"/>
       <c r="P17" t="s">
         <v>309</v>
       </c>
       <c r="Q17" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U17" s="4" t="s">
         <v>25</v>
@@ -3070,23 +3065,23 @@
       </c>
       <c r="H18" s="2"/>
       <c r="I18" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J18" t="s">
+        <v>337</v>
+      </c>
+      <c r="K18" t="s">
         <v>338</v>
       </c>
-      <c r="K18" t="s">
-        <v>339</v>
-      </c>
       <c r="N18" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O18" s="16"/>
       <c r="P18" t="s">
         <v>309</v>
       </c>
       <c r="Q18" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R18" t="s">
         <v>81</v>
@@ -3101,7 +3096,7 @@
         <v>74</v>
       </c>
       <c r="X18" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
@@ -3127,20 +3122,20 @@
         <v>77</v>
       </c>
       <c r="I19" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J19" t="s">
         <v>290</v>
       </c>
       <c r="N19" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O19" s="16"/>
       <c r="P19" t="s">
         <v>309</v>
       </c>
       <c r="Q19" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U19" s="4" t="s">
         <v>25</v>
@@ -3178,23 +3173,23 @@
         <v>86</v>
       </c>
       <c r="I20" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J20" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K20" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>341</v>
-      </c>
       <c r="N20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O20" s="16"/>
       <c r="P20" t="s">
         <v>309</v>
       </c>
       <c r="Q20" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R20" t="s">
         <v>297</v>
@@ -3209,7 +3204,7 @@
         <v>74</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="15.75" x14ac:dyDescent="0.45">
@@ -3236,23 +3231,23 @@
       </c>
       <c r="H21" s="2"/>
       <c r="I21" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J21" t="s">
+        <v>341</v>
+      </c>
+      <c r="K21" t="s">
         <v>342</v>
       </c>
-      <c r="K21" t="s">
-        <v>343</v>
-      </c>
       <c r="N21" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O21" s="16"/>
       <c r="P21" t="s">
         <v>309</v>
       </c>
       <c r="Q21" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R21" t="s">
         <v>73</v>
@@ -3267,7 +3262,7 @@
         <v>74</v>
       </c>
       <c r="X21" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="57" x14ac:dyDescent="0.45">
@@ -3293,27 +3288,27 @@
         <v>77</v>
       </c>
       <c r="I22" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J22" t="s">
+        <v>343</v>
+      </c>
+      <c r="K22" t="s">
         <v>344</v>
-      </c>
-      <c r="K22" t="s">
-        <v>345</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>298</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O22" s="16"/>
       <c r="P22" t="s">
         <v>309</v>
       </c>
       <c r="Q22" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U22" t="s">
         <v>25</v>
@@ -3351,13 +3346,13 @@
         <v>93</v>
       </c>
       <c r="I23" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J23" t="s">
         <v>290</v>
       </c>
       <c r="N23" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O23" s="16"/>
       <c r="P23" t="s">
@@ -3384,13 +3379,13 @@
         <v>13</v>
       </c>
       <c r="I24" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J24" t="s">
         <v>290</v>
       </c>
       <c r="N24" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O24" s="16"/>
       <c r="U24" s="4" t="s">
@@ -3429,13 +3424,13 @@
         <v>99</v>
       </c>
       <c r="I25" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J25" t="s">
         <v>290</v>
       </c>
       <c r="N25" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O25" s="16"/>
       <c r="U25" s="4" t="s">
@@ -3474,13 +3469,13 @@
         <v>99</v>
       </c>
       <c r="I26" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J26" t="s">
         <v>290</v>
       </c>
       <c r="N26" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O26" s="16"/>
       <c r="U26" s="4" t="s">
@@ -3519,13 +3514,13 @@
         <v>105</v>
       </c>
       <c r="I27" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J27" t="s">
         <v>290</v>
       </c>
       <c r="N27" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O27" s="16"/>
       <c r="U27" s="4" t="s">
@@ -3565,13 +3560,13 @@
       </c>
       <c r="H28" s="2"/>
       <c r="I28" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J28" t="s">
         <v>290</v>
       </c>
       <c r="N28" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O28" s="16"/>
       <c r="U28" s="4" t="s">
@@ -3610,13 +3605,13 @@
         <v>111</v>
       </c>
       <c r="I29" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J29" t="s">
         <v>290</v>
       </c>
       <c r="N29" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O29" s="16"/>
       <c r="U29" s="4" t="s">
@@ -3655,13 +3650,13 @@
         <v>114</v>
       </c>
       <c r="I30" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J30" t="s">
         <v>290</v>
       </c>
       <c r="N30" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O30" s="16"/>
       <c r="U30" s="4" t="s">
@@ -3700,13 +3695,13 @@
         <v>117</v>
       </c>
       <c r="I31" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J31" t="s">
         <v>290</v>
       </c>
       <c r="N31" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O31" s="16"/>
       <c r="U31" s="4" t="s">
@@ -3745,13 +3740,13 @@
         <v>120</v>
       </c>
       <c r="I32" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J32" t="s">
         <v>290</v>
       </c>
       <c r="N32" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O32" s="16"/>
       <c r="U32" s="4" t="s">
@@ -3790,13 +3785,13 @@
         <v>120</v>
       </c>
       <c r="I33" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J33" t="s">
         <v>290</v>
       </c>
       <c r="N33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O33" s="16"/>
       <c r="U33" s="4" t="s">
@@ -3835,13 +3830,13 @@
         <v>120</v>
       </c>
       <c r="I34" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J34" t="s">
         <v>290</v>
       </c>
       <c r="N34" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O34" s="16"/>
       <c r="U34" s="4" t="s">
@@ -3880,13 +3875,13 @@
         <v>120</v>
       </c>
       <c r="I35" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J35" t="s">
         <v>290</v>
       </c>
       <c r="N35" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O35" s="16"/>
       <c r="U35" s="4" t="s">
@@ -3925,13 +3920,13 @@
         <v>120</v>
       </c>
       <c r="I36" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J36" t="s">
         <v>290</v>
       </c>
       <c r="N36" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O36" s="16"/>
       <c r="U36" s="4" t="s">
@@ -3970,13 +3965,13 @@
         <v>131</v>
       </c>
       <c r="I37" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J37" t="s">
         <v>290</v>
       </c>
       <c r="N37" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O37" s="16"/>
       <c r="U37" s="4" t="s">
@@ -4016,13 +4011,13 @@
       </c>
       <c r="H38" s="2"/>
       <c r="I38" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J38" t="s">
         <v>290</v>
       </c>
       <c r="N38" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O38" s="16"/>
       <c r="U38" s="4" t="s">
@@ -4061,7 +4056,7 @@
         <v>139</v>
       </c>
       <c r="I39" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J39" t="s">
         <v>290</v>
@@ -4069,7 +4064,7 @@
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
       <c r="N39" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O39" s="16"/>
       <c r="P39"/>
@@ -4113,13 +4108,13 @@
       </c>
       <c r="H40" s="2"/>
       <c r="I40" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J40" t="s">
         <v>290</v>
       </c>
       <c r="N40" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O40" s="16"/>
       <c r="U40" s="4" t="s">
@@ -4158,13 +4153,13 @@
         <v>139</v>
       </c>
       <c r="I41" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J41" t="s">
         <v>290</v>
       </c>
       <c r="N41" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O41" s="16"/>
       <c r="U41" s="4" t="s">
@@ -4203,13 +4198,13 @@
         <v>148</v>
       </c>
       <c r="I42" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J42" t="s">
         <v>290</v>
       </c>
       <c r="N42" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O42" s="16"/>
       <c r="U42" s="4" t="s">
@@ -4249,13 +4244,13 @@
       </c>
       <c r="H43" s="2"/>
       <c r="I43" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J43" t="s">
         <v>290</v>
       </c>
       <c r="N43" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O43" s="16"/>
       <c r="U43" s="4" t="s">
@@ -4294,13 +4289,13 @@
         <v>155</v>
       </c>
       <c r="I44" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J44" t="s">
         <v>290</v>
       </c>
       <c r="N44" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O44" s="16"/>
       <c r="U44" s="4" t="s">
@@ -4339,20 +4334,20 @@
         <v>159</v>
       </c>
       <c r="I45" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J45" t="s">
+        <v>345</v>
+      </c>
+      <c r="K45" t="s">
         <v>346</v>
-      </c>
-      <c r="K45" t="s">
-        <v>347</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>300</v>
       </c>
       <c r="M45" s="5"/>
       <c r="N45" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O45" s="16"/>
       <c r="S45" s="2"/>
@@ -4395,20 +4390,20 @@
         <v>162</v>
       </c>
       <c r="I46" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J46" t="s">
+        <v>347</v>
+      </c>
+      <c r="K46" s="2" t="s">
         <v>348</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>349</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>163</v>
       </c>
       <c r="M46" s="5"/>
       <c r="N46" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O46" s="16"/>
       <c r="U46" t="s">
@@ -4448,27 +4443,27 @@
       </c>
       <c r="H47" s="2"/>
       <c r="I47" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J47" t="s">
+        <v>347</v>
+      </c>
+      <c r="K47" t="s">
         <v>348</v>
-      </c>
-      <c r="K47" t="s">
-        <v>349</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>163</v>
       </c>
       <c r="M47" s="5"/>
       <c r="N47" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O47" s="16"/>
       <c r="P47" t="s">
         <v>309</v>
       </c>
       <c r="Q47" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U47" t="s">
         <v>25</v>
@@ -4480,7 +4475,7 @@
         <v>50</v>
       </c>
       <c r="X47" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="48" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
@@ -4506,27 +4501,27 @@
         <v>169</v>
       </c>
       <c r="I48" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J48" t="s">
+        <v>349</v>
+      </c>
+      <c r="K48" t="s">
         <v>350</v>
-      </c>
-      <c r="K48" t="s">
-        <v>351</v>
       </c>
       <c r="L48" s="5" t="s">
         <v>303</v>
       </c>
       <c r="M48" s="5"/>
       <c r="N48" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O48" s="16"/>
       <c r="P48" t="s">
         <v>309</v>
       </c>
       <c r="Q48" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U48" t="s">
         <v>25</v>
@@ -4538,7 +4533,7 @@
         <v>37</v>
       </c>
       <c r="X48" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="49" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
@@ -4564,27 +4559,27 @@
         <v>173</v>
       </c>
       <c r="I49" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J49" t="s">
+        <v>351</v>
+      </c>
+      <c r="K49" s="2" t="s">
         <v>352</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>353</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>304</v>
       </c>
       <c r="M49" s="5"/>
       <c r="N49" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O49" s="16"/>
       <c r="P49" t="s">
         <v>309</v>
       </c>
       <c r="Q49" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="S49" s="2"/>
       <c r="U49" t="s">
@@ -4597,7 +4592,7 @@
         <v>50</v>
       </c>
       <c r="X49" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="Y49" s="2" t="s">
         <v>305</v>
@@ -4626,27 +4621,27 @@
         <v>173</v>
       </c>
       <c r="I50" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J50" t="s">
+        <v>353</v>
+      </c>
+      <c r="K50" s="2" t="s">
         <v>354</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>355</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>304</v>
       </c>
       <c r="M50" s="5"/>
       <c r="N50" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O50" s="16"/>
       <c r="P50" t="s">
         <v>309</v>
       </c>
       <c r="Q50" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="S50" s="2"/>
       <c r="U50" t="s">
@@ -4659,7 +4654,7 @@
         <v>50</v>
       </c>
       <c r="X50" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="Y50" s="2" t="s">
         <v>305</v>
@@ -4688,27 +4683,27 @@
         <v>173</v>
       </c>
       <c r="I51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J51" t="s">
+        <v>355</v>
+      </c>
+      <c r="K51" t="s">
         <v>356</v>
-      </c>
-      <c r="K51" t="s">
-        <v>357</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>180</v>
       </c>
       <c r="M51" s="5"/>
       <c r="N51" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O51" s="16"/>
       <c r="P51" t="s">
         <v>309</v>
       </c>
       <c r="Q51" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U51" t="s">
         <v>25</v>
@@ -4720,7 +4715,7 @@
         <v>50</v>
       </c>
       <c r="X51" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="52" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
@@ -4746,7 +4741,7 @@
         <v>184</v>
       </c>
       <c r="I52" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J52" t="s">
         <v>290</v>
@@ -4754,7 +4749,7 @@
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
       <c r="N52" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O52" s="16"/>
       <c r="U52" s="4" t="s">
@@ -4793,27 +4788,27 @@
         <v>173</v>
       </c>
       <c r="I53" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J53" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="K53" s="2" t="s">
         <v>358</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>359</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>306</v>
       </c>
       <c r="M53" s="5"/>
       <c r="N53" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O53" s="16"/>
       <c r="P53" t="s">
         <v>309</v>
       </c>
       <c r="Q53" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U53" t="s">
         <v>25</v>
@@ -4825,10 +4820,10 @@
         <v>50</v>
       </c>
       <c r="X53" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="Y53" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="54" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -4854,13 +4849,13 @@
         <v>173</v>
       </c>
       <c r="I54" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J54" t="s">
         <v>290</v>
       </c>
       <c r="N54" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O54" s="16"/>
       <c r="U54" s="4" t="s">
@@ -4899,7 +4894,7 @@
         <v>173</v>
       </c>
       <c r="I55" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J55" t="s">
         <v>290</v>
@@ -4907,7 +4902,7 @@
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
       <c r="N55" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O55" s="16"/>
       <c r="U55" s="4" t="s">
@@ -4946,7 +4941,7 @@
         <v>173</v>
       </c>
       <c r="I56" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J56" t="s">
         <v>290</v>
@@ -4954,7 +4949,7 @@
       <c r="L56" s="5"/>
       <c r="M56" s="5"/>
       <c r="N56" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O56" s="16"/>
       <c r="U56" s="4" t="s">
@@ -4993,13 +4988,13 @@
         <v>173</v>
       </c>
       <c r="I57" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J57" t="s">
         <v>290</v>
       </c>
       <c r="N57" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O57" s="16"/>
       <c r="U57" s="4" t="s">
@@ -5038,13 +5033,13 @@
         <v>173</v>
       </c>
       <c r="I58" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J58" t="s">
         <v>290</v>
       </c>
       <c r="N58" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O58" s="16"/>
       <c r="U58" s="4" t="s">
@@ -5080,13 +5075,13 @@
         <v>16</v>
       </c>
       <c r="I59" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J59" t="s">
         <v>290</v>
       </c>
       <c r="N59" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O59" s="16"/>
       <c r="U59" s="4" t="s">
@@ -5122,13 +5117,13 @@
         <v>16</v>
       </c>
       <c r="I60" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J60" t="s">
         <v>290</v>
       </c>
       <c r="N60" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O60" s="16"/>
       <c r="U60" s="4" t="s">
@@ -5164,13 +5159,13 @@
         <v>16</v>
       </c>
       <c r="I61" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J61" t="s">
         <v>290</v>
       </c>
       <c r="N61" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O61" s="16"/>
       <c r="U61" s="4" t="s">
@@ -5206,13 +5201,13 @@
         <v>16</v>
       </c>
       <c r="I62" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J62" t="s">
         <v>290</v>
       </c>
       <c r="N62" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O62" s="16"/>
       <c r="U62" s="4" t="s">
@@ -5248,13 +5243,13 @@
         <v>16</v>
       </c>
       <c r="I63" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J63" t="s">
         <v>290</v>
       </c>
       <c r="N63" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O63" s="16"/>
       <c r="S63" s="2"/>
@@ -5292,13 +5287,13 @@
         <v>16</v>
       </c>
       <c r="I64" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J64" t="s">
         <v>290</v>
       </c>
       <c r="N64" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O64" s="16"/>
       <c r="U64" s="4" t="s">
@@ -5335,13 +5330,13 @@
       </c>
       <c r="H65" s="2"/>
       <c r="I65" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J65" t="s">
         <v>290</v>
       </c>
       <c r="N65" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O65" s="16"/>
       <c r="U65" s="4" t="s">
@@ -5380,27 +5375,27 @@
         <v>214</v>
       </c>
       <c r="I66" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J66" t="s">
+        <v>359</v>
+      </c>
+      <c r="K66" t="s">
         <v>360</v>
-      </c>
-      <c r="K66" t="s">
-        <v>361</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>306</v>
       </c>
       <c r="M66" s="5"/>
       <c r="N66" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O66" s="16"/>
       <c r="P66" t="s">
         <v>309</v>
       </c>
       <c r="Q66" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="S66" s="2"/>
       <c r="U66" t="s">
@@ -5413,7 +5408,7 @@
         <v>37</v>
       </c>
       <c r="X66" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="Y66" s="2"/>
     </row>
@@ -5441,13 +5436,13 @@
       </c>
       <c r="H67" s="2"/>
       <c r="I67" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J67" t="s">
         <v>290</v>
       </c>
       <c r="N67" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O67" s="16"/>
       <c r="U67" s="4" t="s">
@@ -5486,13 +5481,13 @@
         <v>220</v>
       </c>
       <c r="I68" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J68" t="s">
         <v>290</v>
       </c>
       <c r="N68" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O68" s="16"/>
       <c r="U68" s="4" t="s">
@@ -5531,27 +5526,27 @@
         <v>223</v>
       </c>
       <c r="I69" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J69" t="s">
+        <v>361</v>
+      </c>
+      <c r="K69" s="2" t="s">
         <v>362</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>363</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>307</v>
       </c>
       <c r="M69" s="5"/>
       <c r="N69" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O69" s="16"/>
       <c r="P69" t="s">
         <v>309</v>
       </c>
       <c r="Q69" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U69" t="s">
         <v>25</v>
@@ -5563,7 +5558,7 @@
         <v>50</v>
       </c>
       <c r="X69" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="70" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
@@ -5589,13 +5584,13 @@
         <v>226</v>
       </c>
       <c r="I70" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J70" t="s">
         <v>290</v>
       </c>
       <c r="N70" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O70" s="16"/>
       <c r="U70" s="4" t="s">
@@ -5634,13 +5629,13 @@
         <v>226</v>
       </c>
       <c r="I71" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J71" t="s">
         <v>290</v>
       </c>
       <c r="N71" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O71" s="16"/>
       <c r="U71" s="4" t="s">
@@ -5677,13 +5672,13 @@
       </c>
       <c r="H72" s="2"/>
       <c r="I72" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J72" t="s">
         <v>290</v>
       </c>
       <c r="N72" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O72" s="16"/>
       <c r="U72" s="4" t="s">
@@ -5722,13 +5717,13 @@
         <v>234</v>
       </c>
       <c r="I73" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J73" t="s">
         <v>290</v>
       </c>
       <c r="N73" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O73" s="16"/>
       <c r="U73" s="4" t="s">
@@ -5767,13 +5762,13 @@
         <v>238</v>
       </c>
       <c r="I74" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J74" t="s">
         <v>290</v>
       </c>
       <c r="N74" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O74" s="16"/>
       <c r="U74" s="4" t="s">
@@ -5812,13 +5807,13 @@
         <v>242</v>
       </c>
       <c r="I75" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J75" t="s">
         <v>290</v>
       </c>
       <c r="N75" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O75" s="16"/>
       <c r="U75" s="4" t="s">
@@ -5858,13 +5853,13 @@
       </c>
       <c r="H76" s="2"/>
       <c r="I76" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J76" t="s">
         <v>290</v>
       </c>
       <c r="N76" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O76" s="16"/>
       <c r="S76" s="2"/>
@@ -5905,13 +5900,13 @@
         <v>249</v>
       </c>
       <c r="I77" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J77" t="s">
         <v>290</v>
       </c>
       <c r="N77" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O77" s="16"/>
       <c r="U77" s="4" t="s">
@@ -5950,13 +5945,13 @@
         <v>253</v>
       </c>
       <c r="I78" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J78" t="s">
         <v>290</v>
       </c>
       <c r="N78" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O78" s="16"/>
       <c r="U78" s="4" t="s">
@@ -5995,13 +5990,13 @@
         <v>256</v>
       </c>
       <c r="I79" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J79" t="s">
         <v>290</v>
       </c>
       <c r="N79" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O79" s="16"/>
       <c r="U79" s="4" t="s">
@@ -6040,27 +6035,27 @@
         <v>173</v>
       </c>
       <c r="I80" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J80" t="s">
+        <v>392</v>
+      </c>
+      <c r="K80" t="s">
+        <v>397</v>
+      </c>
+      <c r="L80" s="5" t="s">
         <v>393</v>
-      </c>
-      <c r="K80" t="s">
-        <v>398</v>
-      </c>
-      <c r="L80" s="5" t="s">
-        <v>394</v>
       </c>
       <c r="M80" s="5"/>
       <c r="N80" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="O80" s="16"/>
       <c r="P80" t="s">
         <v>309</v>
       </c>
       <c r="Q80" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="S80" s="2"/>
       <c r="U80" t="s">
@@ -6073,10 +6068,10 @@
         <v>50</v>
       </c>
       <c r="X80" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="Y80" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="81" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
@@ -6102,27 +6097,27 @@
         <v>173</v>
       </c>
       <c r="I81" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J81" t="s">
+        <v>363</v>
+      </c>
+      <c r="K81" t="s">
         <v>364</v>
-      </c>
-      <c r="K81" t="s">
-        <v>365</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>308</v>
       </c>
       <c r="M81" s="5"/>
       <c r="N81" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O81" s="16"/>
       <c r="P81" t="s">
         <v>309</v>
       </c>
       <c r="Q81" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="U81" t="s">
         <v>25</v>
@@ -6134,7 +6129,7 @@
         <v>50</v>
       </c>
       <c r="X81" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="82" spans="1:25" ht="71.25" x14ac:dyDescent="0.45">
@@ -6160,27 +6155,27 @@
         <v>173</v>
       </c>
       <c r="I82" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J82" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="K82" s="6" t="s">
         <v>381</v>
-      </c>
-      <c r="K82" s="6" t="s">
-        <v>382</v>
       </c>
       <c r="L82" s="5"/>
       <c r="M82" s="5" t="s">
         <v>13</v>
       </c>
       <c r="N82" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O82" s="16"/>
       <c r="P82" t="s">
         <v>309</v>
       </c>
       <c r="Q82" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="S82" s="2"/>
       <c r="U82" t="s">
@@ -6196,7 +6191,7 @@
         <v>14</v>
       </c>
       <c r="Y82" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="83" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
@@ -6219,13 +6214,13 @@
         <v>49</v>
       </c>
       <c r="I83" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J83" s="2" t="s">
         <v>290</v>
       </c>
       <c r="N83" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O83" s="16"/>
       <c r="U83" s="4" t="s">
@@ -6264,7 +6259,7 @@
         <v>272</v>
       </c>
       <c r="I84" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J84" s="2" t="s">
         <v>290</v>
@@ -6272,7 +6267,7 @@
       <c r="L84" s="5"/>
       <c r="M84" s="5"/>
       <c r="N84" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O84" s="16"/>
       <c r="U84" s="4" t="s">

</xml_diff>

<commit_message>
r13 correction of body fat percentage
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-NHATS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="160" documentId="8_{B04BC2F6-0886-423B-9CF8-2AF8452D03D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3921F31C-8E7E-479F-8418-8CCBAC8E8062}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{B04BC2F6-0886-423B-9CF8-2AF8452D03D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49363FE2-4286-4BF7-BA46-81E5E7569B2A}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="401">
   <si>
     <t>index</t>
   </si>
@@ -2872,7 +2872,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:25" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>15</v>
       </c>
@@ -3357,6 +3357,18 @@
       <c r="O23" s="16"/>
       <c r="P23" t="s">
         <v>309</v>
+      </c>
+      <c r="U23" t="s">
+        <v>14</v>
+      </c>
+      <c r="V23" t="s">
+        <v>15</v>
+      </c>
+      <c r="W23" t="s">
+        <v>14</v>
+      </c>
+      <c r="X23" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">

</xml_diff>